<commit_message>
Polish pilot copy and sample output
</commit_message>
<xml_diff>
--- a/public/sample/Northstar-Security-Review-Pack.xlsx
+++ b/public/sample/Northstar-Security-Review-Pack.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8c91ed4250f84f69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questionnaire Draft" sheetId="2" r:id="R52186d88e8eb4378"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Answers" sheetId="3" r:id="R18e350d54b9a4399"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="4" r:id="R4da0dafd00b54137"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Register" sheetId="5" r:id="Rd78f2508c5864769"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R13f9a0f388124ad3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questionnaire Draft" sheetId="2" r:id="R99b3d522e7704888"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approved Answers" sheetId="3" r:id="Rf5c32bffb5a042aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="4" r:id="R04171d917dea463d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Register" sheetId="5" r:id="R1de23c51b1634392"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -729,7 +729,7 @@
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ApprovedAnswerTable" displayName="ApprovedAnswerTable" ref="A5:H9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Claim ID"/>
-    <x:tableColumn id="2" name="Question pattern"/>
+    <x:tableColumn id="2" name="Claim / topic"/>
     <x:tableColumn id="3" name="Approved answer"/>
     <x:tableColumn id="4" name="Evidence IDs"/>
     <x:tableColumn id="5" name="Evidence owners"/>
@@ -1342,9 +1342,7 @@
         <x:v>NS-EV-001</x:v>
       </x:c>
       <x:c r="G6" s="26" t="str"/>
-      <x:c r="H6" s="26" t="str">
-        <x:v>Customer owner must verify.</x:v>
-      </x:c>
+      <x:c r="H6" s="26" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="27" t="str">
@@ -1366,9 +1364,7 @@
         <x:v>NS-EV-002</x:v>
       </x:c>
       <x:c r="G7" s="27" t="str"/>
-      <x:c r="H7" s="27" t="str">
-        <x:v>Customer owner must verify.</x:v>
-      </x:c>
+      <x:c r="H7" s="27" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="27" t="str">
@@ -1390,9 +1386,7 @@
         <x:v>NS-EV-002</x:v>
       </x:c>
       <x:c r="G8" s="27" t="str"/>
-      <x:c r="H8" s="27" t="str">
-        <x:v>Customer owner must verify.</x:v>
-      </x:c>
+      <x:c r="H8" s="27" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="27" t="str">
@@ -1414,10 +1408,10 @@
         <x:v>NS-EV-001;NS-EV-002</x:v>
       </x:c>
       <x:c r="G9" s="27" t="str">
-        <x:v>conflict regex matched NS-EV-002: (?i)15 minutes of inactivity</x:v>
+        <x:v>Available sources do not support one clear, current answer.</x:v>
       </x:c>
       <x:c r="H9" s="27" t="str">
-        <x:v>Resolve the conflicting evidence and approve a single current source.</x:v>
+        <x:v>Reconcile the available sources and confirm one current answer.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1440,10 +1434,10 @@
         <x:v>NS-EV-003</x:v>
       </x:c>
       <x:c r="G10" s="27" t="str">
-        <x:v>evidence NS-EV-003 is not current: evidence status is not approved; evidence expired on 2025-01-15; evidence is older than 365 days; conflict regex matched NS-EV-003: (?i)has not been reapproved</x:v>
+        <x:v>The supporting evidence is outdated or no longer approved.</x:v>
       </x:c>
       <x:c r="H10" s="27" t="str">
-        <x:v>Resolve the conflicting evidence and approve a single current source.</x:v>
+        <x:v>Replace or reapprove the outdated source, then confirm the answer.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1466,9 +1460,7 @@
         <x:v>NS-EV-004</x:v>
       </x:c>
       <x:c r="G11" s="27" t="str"/>
-      <x:c r="H11" s="27" t="str">
-        <x:v>Customer owner must verify.</x:v>
-      </x:c>
+      <x:c r="H11" s="27" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="27" t="str">
@@ -1488,10 +1480,10 @@
       </x:c>
       <x:c r="F12" s="27" t="str"/>
       <x:c r="G12" s="27" t="str">
-        <x:v>no explicit approved claim matches this question</x:v>
+        <x:v>No approved, evidence-backed answer is available for this question.</x:v>
       </x:c>
       <x:c r="H12" s="27" t="str">
-        <x:v>Add an explicitly approved claim with current evidence for this question.</x:v>
+        <x:v>Provide and approve current evidence for this question.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1512,10 +1504,10 @@
       </x:c>
       <x:c r="F13" s="28" t="str"/>
       <x:c r="G13" s="28" t="str">
-        <x:v>no explicit approved claim matches this question</x:v>
+        <x:v>No approved, evidence-backed answer is available for this question.</x:v>
       </x:c>
       <x:c r="H13" s="28" t="str">
-        <x:v>Add an explicitly approved claim with current evidence for this question.</x:v>
+        <x:v>Provide and approve current evidence for this question.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1532,7 +1524,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R397943adccfd418a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76b45b0d580e4cc0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1590,7 +1582,7 @@
         <x:v>Claim ID</x:v>
       </x:c>
       <x:c r="B5" s="17" t="str">
-        <x:v>Question pattern</x:v>
+        <x:v>Claim / topic</x:v>
       </x:c>
       <x:c r="C5" s="17" t="str">
         <x:v>Approved answer</x:v>
@@ -1616,7 +1608,7 @@
         <x:v>departing-user-disablement</x:v>
       </x:c>
       <x:c r="B6" s="26" t="str">
-        <x:v>(?i)departing users.{0,80}disabled.{0,40}24 hours</x:v>
+        <x:v>Departing user account disablement</x:v>
       </x:c>
       <x:c r="C6" s="26" t="str">
         <x:v>Accounts belonging to departing users are disabled within 24 hours of the recorded departure time.</x:v>
@@ -1642,7 +1634,7 @@
         <x:v>privileged-mfa</x:v>
       </x:c>
       <x:c r="B7" s="27" t="str">
-        <x:v>(?i)privileged accounts.{0,80}multi-factor authentication</x:v>
+        <x:v>Privileged account multi-factor authentication</x:v>
       </x:c>
       <x:c r="C7" s="27" t="str">
         <x:v>All privileged accounts are protected by multi-factor authentication.</x:v>
@@ -1668,7 +1660,7 @@
         <x:v>security-policy-current</x:v>
       </x:c>
       <x:c r="B8" s="27" t="str">
-        <x:v>(?i)information security policy</x:v>
+        <x:v>Current information security policy</x:v>
       </x:c>
       <x:c r="C8" s="27" t="str">
         <x:v>Northstar maintains a formally approved information security policy that is reviewed at least annually.</x:v>
@@ -1694,7 +1686,7 @@
         <x:v>subprocessor-register-current</x:v>
       </x:c>
       <x:c r="B9" s="28" t="str">
-        <x:v>(?i)(?:inventory|register).{0,80}subprocessors</x:v>
+        <x:v>Current subprocessor register</x:v>
       </x:c>
       <x:c r="C9" s="28" t="str">
         <x:v>Northstar maintains a current subprocessor register containing each provider's processing purpose and region.</x:v>
@@ -1729,7 +1721,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra958ce54293944d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R526a39cc44da4477"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1907,7 +1899,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bda08f4bceb4411"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84f6327a89fa4756"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1973,10 +1965,10 @@
         <x:v>What inactivity timeout is enforced for administrator sessions?</x:v>
       </x:c>
       <x:c r="C6" s="26" t="str">
-        <x:v>conflict regex matched NS-EV-002: (?i)15 minutes of inactivity</x:v>
+        <x:v>Available sources do not support one clear, current answer.</x:v>
       </x:c>
       <x:c r="D6" s="26" t="str">
-        <x:v>Resolve the conflicting evidence and approve a single current source.</x:v>
+        <x:v>Reconcile the available sources and confirm one current answer.</x:v>
       </x:c>
       <x:c r="E6" s="26" t="str">
         <x:v>conflicting</x:v>
@@ -1990,10 +1982,10 @@
         <x:v>Does the organisation maintain a current, approved incident response plan?</x:v>
       </x:c>
       <x:c r="C7" s="27" t="str">
-        <x:v>evidence NS-EV-003 is not current: evidence status is not approved; evidence expired on 2025-01-15; evidence is older than 365 days; conflict regex matched NS-EV-003: (?i)has not been reapproved</x:v>
+        <x:v>The supporting evidence is outdated or no longer approved.</x:v>
       </x:c>
       <x:c r="D7" s="27" t="str">
-        <x:v>Resolve the conflicting evidence and approve a single current source.</x:v>
+        <x:v>Replace or reapprove the outdated source, then confirm the answer.</x:v>
       </x:c>
       <x:c r="E7" s="27" t="str">
         <x:v>conflicting</x:v>
@@ -2007,10 +1999,10 @@
         <x:v>Has an independent penetration test been completed within the last 12 months?</x:v>
       </x:c>
       <x:c r="C8" s="27" t="str">
-        <x:v>no explicit approved claim matches this question</x:v>
+        <x:v>No approved, evidence-backed answer is available for this question.</x:v>
       </x:c>
       <x:c r="D8" s="27" t="str">
-        <x:v>Add an explicitly approved claim with current evidence for this question.</x:v>
+        <x:v>Provide and approve current evidence for this question.</x:v>
       </x:c>
       <x:c r="E8" s="27" t="str">
         <x:v>unsupported</x:v>
@@ -2024,10 +2016,10 @@
         <x:v>Does the organisation hold a current SOC 2 Type II report?</x:v>
       </x:c>
       <x:c r="C9" s="28" t="str">
-        <x:v>no explicit approved claim matches this question</x:v>
+        <x:v>No approved, evidence-backed answer is available for this question.</x:v>
       </x:c>
       <x:c r="D9" s="28" t="str">
-        <x:v>Add an explicitly approved claim with current evidence for this question.</x:v>
+        <x:v>Provide and approve current evidence for this question.</x:v>
       </x:c>
       <x:c r="E9" s="28" t="str">
         <x:v>unsupported</x:v>
@@ -2047,7 +2039,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b34b176f1764774"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9eaa8589a9e84fc3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>